<commit_message>
fix(stock): remove custom unquoted currency style format in xlsx generation to fix MS Excel XML repair warning
</commit_message>
<xml_diff>
--- a/frontend/static/Insumos_15_Ejemplo_VitaMetrix.xlsx
+++ b/frontend/static/Insumos_15_Ejemplo_VitaMetrix.xlsx
@@ -16,9 +16,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="Bs#,##0.00"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -89,7 +87,7 @@
     <xf numFmtId="3" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -460,16 +458,16 @@
   <dimension ref="A1:M16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="71" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="56" customWidth="1" min="2" max="2"/>
     <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="29" customWidth="1" min="5" max="5"/>
-    <col width="25" customWidth="1" min="6" max="6"/>
-    <col width="21" customWidth="1" min="7" max="7"/>
-    <col width="27" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="24" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="17" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
     <col width="28" customWidth="1" min="11" max="11"/>
     <col width="28" customWidth="1" min="12" max="12"/>
     <col width="59" customWidth="1" min="13" max="13"/>
@@ -478,67 +476,67 @@
     <row r="1" ht="28" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>CÓDIGO / SKU</t>
+          <t>SKU</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>NOMBRE PRODUCTO / INSUMO*</t>
+          <t>Nombre Producto / Insumo*</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>CATEGORÍA</t>
+          <t>Categoría</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>UNIDAD DE MEDIDA</t>
+          <t>U. Medida</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>CANTIDAD INICIAL (STOCK)*</t>
+          <t>Stock*</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>STOCK MÍNIMO (ALERTA)</t>
+          <t>St. Min</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>PRECIO COSTO (BS)</t>
+          <t>P. Costo (Bs)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>PRECIO VENTA / PVP (BS)</t>
+          <t>PVP (Bs)</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>NÚMERO DE LOTE</t>
+          <t>Lote</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>FECHA DE VENCIMIENTO</t>
+          <t>Vencimiento</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>UBICACIÓN EN CONSULTORIO</t>
+          <t>Ubicación</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>PROVEEDOR</t>
+          <t>Proveedor</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>NOTAS / POSOLOGÍA</t>
+          <t>Notas / Posología</t>
         </is>
       </c>
     </row>
@@ -786,7 +784,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Multivitamínico Clínico Complejo B + ZINC (Caja x60 Cápsulas)</t>
+          <t>Multivitamínico Clínico Complejo B + ZINC (Caja x60)</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -845,7 +843,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Omega 3 Ultra Purificado 1000mg (Frasco x120 Perlas)</t>
+          <t>Omega 3 Ultra Purificado 1000mg (Frasco x120)</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
@@ -1140,7 +1138,7 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Cálper / Plicómetro Antropométrico Clínico Slimguide</t>
+          <t>Cálper / Plicómetro Antropométrico Slimguide</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
@@ -1376,7 +1374,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Fórmulas Magistrales Inyectables Complejo Vitamínico (Ampollas x10)</t>
+          <t>Fórmulas Magistrales Inyectables Complejo Vitamínico</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">

</xml_diff>

<commit_message>
feat(excel): standardize 13-column Excel template headers and parsing logic matching P. Costo (Bs), PVP (Bs) and Notas / Posologia
</commit_message>
<xml_diff>
--- a/frontend/static/Insumos_15_Ejemplo_VitaMetrix.xlsx
+++ b/frontend/static/Insumos_15_Ejemplo_VitaMetrix.xlsx
@@ -459,8 +459,8 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="56" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="51" customWidth="1" min="2" max="2"/>
+    <col width="29" customWidth="1" min="3" max="3"/>
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
@@ -468,9 +468,9 @@
     <col width="14" customWidth="1" min="8" max="8"/>
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="15" customWidth="1" min="10" max="10"/>
-    <col width="28" customWidth="1" min="11" max="11"/>
+    <col width="25" customWidth="1" min="11" max="11"/>
     <col width="28" customWidth="1" min="12" max="12"/>
-    <col width="59" customWidth="1" min="13" max="13"/>
+    <col width="54" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -654,7 +654,7 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>Conservar en lugar fresco y fuera de luz solar</t>
+          <t>Conservar en lugar fresco</t>
         </is>
       </c>
     </row>
@@ -784,7 +784,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Multivitamínico Clínico Complejo B + ZINC (Caja x60)</t>
+          <t>Multivitamínico Clínico Complejo B + ZINC</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
@@ -843,54 +843,54 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Omega 3 Ultra Purificado 1000mg (Frasco x120)</t>
+          <t>Toallitas de Alcohol Isopropílico 70%</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Suplementos Nutricionales</t>
+          <t>Material Clínico</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Frasco</t>
+          <t>Caja x200</t>
         </is>
       </c>
       <c r="E7" s="3" t="n">
-        <v>14</v>
+        <v>30</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>110</v>
+        <v>35</v>
       </c>
       <c r="H7" s="4" t="n">
-        <v>165</v>
+        <v>55</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>OMG-554</t>
+          <t>ALC-2026-X</t>
         </is>
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>2027-08-18</t>
+          <t>2029-01-01</t>
         </is>
       </c>
       <c r="K7" s="2" t="inlineStr">
         <is>
-          <t>Vitrina 2, Cajón A</t>
+          <t>Mesa de Examen</t>
         </is>
       </c>
       <c r="L7" s="2" t="inlineStr">
         <is>
-          <t>PharmaLife S.A.</t>
+          <t>BioMedical Import S.R.L.</t>
         </is>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>Concentrado de EPA 500mg / DHA 250mg</t>
+          <t>Limpieza previa a bioimpedancia</t>
         </is>
       </c>
     </row>
@@ -902,54 +902,50 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Toallitas de Alcohol Isopropílico 70% (Caja x200)</t>
+          <t>Cinta Métrica Antropométrica Lufkin</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Material Clínico e Higiene</t>
+          <t>Accesorios</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Caja x200</t>
+          <t>Unidad</t>
         </is>
       </c>
       <c r="E8" s="3" t="n">
-        <v>30</v>
+        <v>8</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>35</v>
+        <v>95</v>
       </c>
       <c r="H8" s="4" t="n">
-        <v>55</v>
+        <v>140</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>ALC-991</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="inlineStr">
-        <is>
-          <t>2029-01-01</t>
-        </is>
-      </c>
+          <t>LUF-991</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr"/>
       <c r="K8" s="2" t="inlineStr">
         <is>
-          <t>Mesa de Examen</t>
+          <t>Gabinete 2</t>
         </is>
       </c>
       <c r="L8" s="2" t="inlineStr">
         <is>
-          <t>Dispromed Bolivia</t>
+          <t>NutriFit Express</t>
         </is>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>Desinfección de electrodos y piel pre-BIA</t>
+          <t>Calibrada en milímetros</t>
         </is>
       </c>
     </row>
@@ -961,54 +957,50 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Guantes de Nitrilo Examen Talla M (Caja x100)</t>
+          <t>Plicómetro Antropométrico Harpenden</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Material Clínico e Higiene</t>
+          <t>Accesorios</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Caja x100</t>
+          <t>Unidad</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
-        <v>22</v>
+        <v>3</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>45</v>
+        <v>1200</v>
       </c>
       <c r="H9" s="4" t="n">
-        <v>70</v>
+        <v>1600</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>GLV-2026-M</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="inlineStr">
-        <is>
-          <t>2028-10-30</t>
-        </is>
-      </c>
+          <t>HARP-012</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr"/>
       <c r="K9" s="2" t="inlineStr">
         <is>
-          <t>Mesa de Examen</t>
+          <t>Gabinete 2</t>
         </is>
       </c>
       <c r="L9" s="2" t="inlineStr">
         <is>
-          <t>Dispromed Bolivia</t>
+          <t>Equipos Médicos S.R.L.</t>
         </is>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>Libre de látex y talco</t>
+          <t>Presión constante de 10g/mm2</t>
         </is>
       </c>
     </row>
@@ -1020,54 +1012,54 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Papel Camilla Desechable 50cm x 100m (Rollo)</t>
+          <t>Omega 3 Concentrado EPA/DHA 1000mg</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Material Clínico e Higiene</t>
+          <t>Suplementos Nutricionales</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Rollo</t>
+          <t>Frasco x120</t>
         </is>
       </c>
       <c r="E10" s="3" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>60</v>
+        <v>150</v>
       </c>
       <c r="H10" s="4" t="n">
-        <v>90</v>
+        <v>220</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>PPL-401</t>
+          <t>OMG-771</t>
         </is>
       </c>
       <c r="J10" s="2" t="inlineStr">
         <is>
-          <t>2030-01-01</t>
+          <t>2027-10-01</t>
         </is>
       </c>
       <c r="K10" s="2" t="inlineStr">
         <is>
-          <t>Almacén Inferior Camilla</t>
+          <t>Estante B</t>
         </is>
       </c>
       <c r="L10" s="2" t="inlineStr">
         <is>
-          <t>Dispromed Bolivia</t>
+          <t>PharmaLife S.A.</t>
         </is>
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>Protección de camilla de bioimpedancia</t>
+          <t>2 cápsulas con comidas</t>
         </is>
       </c>
     </row>
@@ -1079,54 +1071,54 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Cinta Métrica Antropométrica Ergonómica Seca 201</t>
+          <t>Magnesio Citrato 500mg Polvo</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Accesorios y Equipos</t>
+          <t>Suplementos Nutricionales</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Unidad (u)</t>
+          <t>Frasco 250g</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="H11" s="4" t="n">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>EQ-SECA-01</t>
+          <t>MAG-330</t>
         </is>
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>2035-12-31</t>
+          <t>2027-05-14</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr">
         <is>
-          <t>Estuche Antropométrico</t>
+          <t>Estante B</t>
         </is>
       </c>
       <c r="L11" s="2" t="inlineStr">
         <is>
-          <t>Seca Medical Equipment</t>
+          <t>PharmaLife S.A.</t>
         </is>
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>Medición de perímetro abdominal y cintura</t>
+          <t>Disolver 1 medida en agua por las noches</t>
         </is>
       </c>
     </row>
@@ -1138,54 +1130,54 @@
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Cálper / Plicómetro Antropométrico Slimguide</t>
+          <t>Colágeno Hidrolizado + Vitamina C</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Accesorios y Equipos</t>
+          <t>Suplementos Nutricionales</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Unidad (u)</t>
+          <t>Bote 500g</t>
         </is>
       </c>
       <c r="E12" s="3" t="n">
-        <v>4</v>
+        <v>16</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="G12" s="4" t="n">
-        <v>130</v>
+        <v>180</v>
       </c>
       <c r="H12" s="4" t="n">
-        <v>190</v>
+        <v>260</v>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
-          <t>EQ-SLIM-04</t>
+          <t>COL-909</t>
         </is>
       </c>
       <c r="J12" s="2" t="inlineStr">
         <is>
-          <t>2035-12-31</t>
+          <t>2027-07-22</t>
         </is>
       </c>
       <c r="K12" s="2" t="inlineStr">
         <is>
-          <t>Estuche Antropométrico</t>
+          <t>Estante A</t>
         </is>
       </c>
       <c r="L12" s="2" t="inlineStr">
         <is>
-          <t>Seca Medical Equipment</t>
+          <t>NutriFit Express</t>
         </is>
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>Medición de pliegues cutáneos tricipital y subescapular</t>
+          <t>Tomar en ayunas</t>
         </is>
       </c>
     </row>
@@ -1197,54 +1189,54 @@
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Tiras Reactivas para Examen de Orina (Frasco x100)</t>
+          <t>L-Carnitina Liquida 3000mg</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Material Clínico e Higiene</t>
+          <t>Suplementos Nutricionales</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Frasco</t>
+          <t>Frasco 500ml</t>
         </is>
       </c>
       <c r="E13" s="3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>3</v>
       </c>
       <c r="G13" s="4" t="n">
-        <v>75</v>
+        <v>110</v>
       </c>
       <c r="H13" s="4" t="n">
-        <v>115</v>
+        <v>165</v>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
-          <t>URI-330</t>
+          <t>LCAR-909</t>
         </is>
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>2027-05-14</t>
+          <t>2027-07-22</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr">
         <is>
-          <t>Vitrina 2, Cajón C</t>
+          <t>Estante A</t>
         </is>
       </c>
       <c r="L13" s="2" t="inlineStr">
         <is>
-          <t>BioLab Diagnósticos</t>
+          <t>NutriFit Express</t>
         </is>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>Evaluación rápida de densidad e hidratación</t>
+          <t>Tomar 15ml antes del entrenamiento</t>
         </is>
       </c>
     </row>
@@ -1256,7 +1248,7 @@
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Colágeno Hidrolizado + Ácido Hialurónico 500g</t>
+          <t>Aminoácidos BCAA 2:1:1 Polvo</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
@@ -1266,34 +1258,34 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Bote 500g</t>
+          <t>Bote 400g</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F14" s="3" t="n">
         <v>4</v>
       </c>
       <c r="G14" s="4" t="n">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="H14" s="4" t="n">
-        <v>260</v>
+        <v>275</v>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>COL-771</t>
+          <t>BCAA-2026</t>
         </is>
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>2027-10-01</t>
+          <t>2027-08-30</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr">
         <is>
-          <t>Estante Suplementos B</t>
+          <t>Estante A</t>
         </is>
       </c>
       <c r="L14" s="2" t="inlineStr">
@@ -1303,7 +1295,7 @@
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>Salud articular y firmeza de tejidos</t>
+          <t>Intra-entrenamiento</t>
         </is>
       </c>
     </row>
@@ -1315,54 +1307,54 @@
       </c>
       <c r="B15" s="2" t="inlineStr">
         <is>
-          <t>L-Carnitina 3000mg Líquida (Frasco 500ml Manzana)</t>
+          <t>Guantes de Nitrilo Desechables Talla M</t>
         </is>
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Suplementos Nutricionales</t>
+          <t>Material Clínico</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>Frasco 500ml</t>
+          <t>Caja x100</t>
         </is>
       </c>
       <c r="E15" s="3" t="n">
-        <v>12</v>
+        <v>40</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>3</v>
+        <v>10</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>140</v>
+        <v>45</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>195</v>
+        <v>70</v>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
-          <t>LCAR-909</t>
+          <t>NIT-2026</t>
         </is>
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>2027-07-22</t>
+          <t>2029-05-01</t>
         </is>
       </c>
       <c r="K15" s="2" t="inlineStr">
         <is>
-          <t>Estante Suplementos B</t>
+          <t>Mesa de Examen</t>
         </is>
       </c>
       <c r="L15" s="2" t="inlineStr">
         <is>
-          <t>NutriFit Express</t>
+          <t>DermoSalud Bolivia</t>
         </is>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>Tomar 15ml antes del entrenamiento</t>
+          <t>Libres de polvo</t>
         </is>
       </c>
     </row>
@@ -1374,54 +1366,54 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Fórmulas Magistrales Inyectables Complejo Vitamínico</t>
+          <t>Mascarillas Quirúrgicas 3 Capas</t>
         </is>
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Medicamentos / Fármacos</t>
+          <t>Material Clínico</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Caja x10</t>
+          <t>Caja x50</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="F16" s="3" t="n">
         <v>10</v>
       </c>
-      <c r="F16" s="3" t="n">
-        <v>2</v>
-      </c>
       <c r="G16" s="4" t="n">
-        <v>210</v>
+        <v>20</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>310</v>
+        <v>35</v>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>AMP-2026-X</t>
+          <t>MAS-100</t>
         </is>
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>2027-06-30</t>
+          <t>2029-12-31</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr">
         <is>
-          <t>Refrigerador Clínico</t>
+          <t>Mesa de Examen</t>
         </is>
       </c>
       <c r="L16" s="2" t="inlineStr">
         <is>
-          <t>Magistra Lab S.R.L.</t>
+          <t>DermoSalud Bolivia</t>
         </is>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>Mantener refrigerado entre 2°C y 8°C</t>
+          <t>Eficiencia de filtración &gt; 95%</t>
         </is>
       </c>
     </row>

</xml_diff>